<commit_message>
Commit_Update_Agent Module_Ops Module_DMC Module part
</commit_message>
<xml_diff>
--- a/server/uploads/1782120985355-transport_usage_type_distinct_rates_colored_fixed.xlsx
+++ b/server/uploads/1782120985355-transport_usage_type_distinct_rates_colored_fixed.xlsx
@@ -1509,8 +1509,8 @@
       <c r="G17" t="str">
         <v/>
       </c>
-      <c r="H17" t="str">
-        <v>Point To Point</v>
+      <c r="H17">
+        <v>2100</v>
       </c>
       <c r="I17" t="str">
         <v/>
@@ -30069,8 +30069,8 @@
       <c r="G437" t="str">
         <v/>
       </c>
-      <c r="H437" t="str">
-        <v>Point To Point</v>
+      <c r="H437">
+        <v>4650</v>
       </c>
       <c r="I437" t="str">
         <v/>

</xml_diff>